<commit_message>
US spelling throughout (color, labeled, gray, judgment)
</commit_message>
<xml_diff>
--- a/output/Retail_Peer_Benchmarking.xlsx
+++ b/output/Retail_Peer_Benchmarking.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\competitor-scorecard\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\retail-peer-benchmarking\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B931D4A3-71EC-46CC-8F7B-3CFD886D877E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D723968E-169C-4CC6-90A0-42D6D11B2036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -209,7 +209,7 @@
     <t>Units</t>
   </si>
   <si>
-    <t>USD millions unless stated; fiscal years labelled by SEC frame convention (see Methodology)</t>
+    <t>USD millions unless stated; fiscal years labeled by SEC frame convention (see Methodology)</t>
   </si>
   <si>
     <t>Status</t>
@@ -353,7 +353,7 @@
     <t>RETAIL PEER BENCHMARKING   ·   FY2016–FY2025   ·   SEC 10-K DATA</t>
   </si>
   <si>
-    <t>As reported in SEC 10-K filings. USD millions. Blue = hard-coded input from EDGAR XBRL (one citation per value on the Data Lineage tab); black = formula; 'n/a' = not reported – flagged, never estimated. Fiscal years labelled by SEC frame convention (FY2025 = Walmart fiscal 2026, Kroger 2025, Costco 2025).</t>
+    <t>As reported in SEC 10-K filings. USD millions. Blue = hard-coded input from EDGAR XBRL (one citation per value on the Data Lineage tab); black = formula; 'n/a' = not reported – flagged, never estimated. Fiscal years labeled by SEC frame convention (FY2025 = Walmart fiscal 2026, Kroger 2025, Costco 2025).</t>
   </si>
   <si>
     <t>Line item</t>
@@ -746,7 +746,7 @@
     <t>2025-10-08</t>
   </si>
   <si>
-    <t>Legend: blue = SEC input · black bold = formula · shaded yellow = value taken from the XBRL instance document or derived from two tagged facts (see note) · grey band = debt-build components · 'n/a' = not reported.</t>
+    <t>Legend: blue = SEC input · black bold = formula · shaded yellow = value taken from the XBRL instance document or derived from two tagged facts (see note) · gray band = debt-build components · 'n/a' = not reported.</t>
   </si>
   <si>
     <t>04   —   RATIO CALCULATIONS</t>
@@ -812,7 +812,7 @@
     <t>05   —   SCORECARD</t>
   </si>
   <si>
-    <t>Direction-aware ranks and colour scales (green = strongest) · change the year to re-rank</t>
+    <t>Direction-aware ranks and color scales (green = strongest) · change the year to re-rank</t>
   </si>
   <si>
     <t>Scorecard year (input)</t>
@@ -956,7 +956,7 @@
     <t>XLOOKUP + IFERROR</t>
   </si>
   <si>
-    <t>All ratio cells: =IFERROR((XLOOKUP(year,Years,Company_Revenue)-XLOOKUP(year,Years,Company_COGS))/XLOOKUP(year,Years,Company_Revenue),"n/a"). Missing data returns the text n/a rather than #DIV/0! or #VALUE!, and is styled grey-italic by conditional formatting.</t>
+    <t>All ratio cells: =IFERROR((XLOOKUP(year,Years,Company_Revenue)-XLOOKUP(year,Years,Company_COGS))/XLOOKUP(year,Years,Company_Revenue),"n/a"). Missing data returns the text n/a rather than #DIV/0! or #VALUE!, and is styled gray-italic by conditional formatting.</t>
   </si>
   <si>
     <t>Formula-built totals</t>
@@ -968,13 +968,13 @@
     <t>Scorecard year input</t>
   </si>
   <si>
-    <t>Data-validated list (FY2016–FY2025) driving XLOOKUPs on the Scorecard and the at-a-glance figures; ranks and colour scales recompute.</t>
+    <t>Data-validated list (FY2016–FY2025) driving XLOOKUPs on the Scorecard and the at-a-glance figures; ranks and color scales recompute.</t>
   </si>
   <si>
     <t>Conditional formatting</t>
   </si>
   <si>
-    <t>Three-colour scales per metric row (direction-aware: low debt-to-equity is green), text-detection rules for n/a, and a reversed scale on the composite rank.</t>
+    <t>Three-color scales per metric row (direction-aware: low debt-to-equity is green), text-detection rules for n/a, and a reversed scale on the composite rank.</t>
   </si>
   <si>
     <t>Native combo charts</t>
@@ -986,7 +986,7 @@
     <t>Model conventions</t>
   </si>
   <si>
-    <t>Blue font = hard-coded SEC input; black = formula; yellow shading = instance/derived value; grey band = debt components; freeze panes, print titles, fit-to-width and footers on every tab; document properties set.</t>
+    <t>Blue font = hard-coded SEC input; black = formula; yellow shading = instance/derived value; gray band = debt components; freeze panes, print titles, fit-to-width and footers on every tab; document properties set.</t>
   </si>
   <si>
     <t>Verification</t>
@@ -1019,7 +1019,7 @@
     <t>Inventory (LIFO vs FIFO)</t>
   </si>
   <si>
-    <t>Walmart U.S. (retail method, LIFO), Sam's Club (weighted-average, LIFO), Costco U.S. (LIFO), Kroger (~91% LIFO, link-chain dollar-value) and Whole Foods (LIFO) all report cost of sales after a LIFO charge in inflationary years; Costco Canada and Walmart International are FIFO. In 2021–2023 LIFO raised reported cost of sales and depressed gross margin and inventory for the LIFO filers – Kroger's reserve grew from $1.3B (FY2016) to $2.6B (FY2025) and its LIFO charge was $157M in FY2025; Costco's FY2022 LIFO charge cost 19 bp of gross margin (~$0.4B), FY2023–FY2024 were immaterial, FY2025 7 bp. Effects: (a) gross margins for FY2021–FY2023 are understated relative to a FIFO basis, more so for Kroger; (b) current assets and therefore the current ratio are understated for LIFO filers; (c) only Kroger discloses a reserve balance – Walmart stated that LIFO approximated FIFO through January 2022 (FY2021) and has given only sensitivity language since; Costco discloses the annual charge but no reserve balance. Ratios are presented as reported and trends, rather than levels, are emphasised in the findings.</t>
+    <t>Walmart U.S. (retail method, LIFO), Sam's Club (weighted-average, LIFO), Costco U.S. (LIFO), Kroger (~91% LIFO, link-chain dollar-value) and Whole Foods (LIFO) all report cost of sales after a LIFO charge in inflationary years; Costco Canada and Walmart International are FIFO. In 2021–2023 LIFO raised reported cost of sales and depressed gross margin and inventory for the LIFO filers – Kroger's reserve grew from $1.3B (FY2016) to $2.6B (FY2025) and its LIFO charge was $157M in FY2025; Costco's FY2022 LIFO charge cost 19 bp of gross margin (~$0.4B), FY2023–FY2024 were immaterial, FY2025 7 bp. Effects: (a) gross margins for FY2021–FY2023 are understated relative to a FIFO basis, more so for Kroger; (b) current assets and therefore the current ratio are understated for LIFO filers; (c) only Kroger discloses a reserve balance – Walmart stated that LIFO approximated FIFO through January 2022 (FY2021) and has given only sensitivity language since; Costco discloses the annual charge but no reserve balance. Ratios are presented as reported and trends, rather than levels, are emphasized in the findings.</t>
   </si>
   <si>
     <t>Equity and net income</t>
@@ -1046,7 +1046,7 @@
     <t>Assumptions</t>
   </si>
   <si>
-    <t>Latest-filed values are the best available (restatements are accepted); segment operating income is comparable to consolidated operating income for margin purposes; Amazon 'Physical stores' is used as a revenue proxy for Whole Foods and labelled as such.</t>
+    <t>Latest-filed values are the best available (restatements are accepted); segment operating income is comparable to consolidated operating income for margin purposes; Amazon 'Physical stores' is used as a revenue proxy for Whole Foods and labeled as such.</t>
   </si>
   <si>
     <t>Out of scope</t>
@@ -2667,7 +2667,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-58A9-408C-84E7-B3658E346BA1}"/>
+              <c16:uniqueId val="{00000000-7887-4E4E-9E06-D69A0794FE8C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2680,8 +2680,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1461336879"/>
-        <c:axId val="874278767"/>
+        <c:axId val="1442829296"/>
+        <c:axId val="1377578992"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2803,7 +2803,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-58A9-408C-84E7-B3658E346BA1}"/>
+              <c16:uniqueId val="{00000001-7887-4E4E-9E06-D69A0794FE8C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2924,7 +2924,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-58A9-408C-84E7-B3658E346BA1}"/>
+              <c16:uniqueId val="{00000002-7887-4E4E-9E06-D69A0794FE8C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3045,7 +3045,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-58A9-408C-84E7-B3658E346BA1}"/>
+              <c16:uniqueId val="{00000003-7887-4E4E-9E06-D69A0794FE8C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3166,7 +3166,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-58A9-408C-84E7-B3658E346BA1}"/>
+              <c16:uniqueId val="{00000004-7887-4E4E-9E06-D69A0794FE8C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3287,7 +3287,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-58A9-408C-84E7-B3658E346BA1}"/>
+              <c16:uniqueId val="{00000005-7887-4E4E-9E06-D69A0794FE8C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3364,7 +3364,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="874278767"/>
+        <c:axId val="1377578992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3399,12 +3399,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1461336879"/>
+        <c:crossAx val="1442829296"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1461336879"/>
+        <c:axId val="1442829296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3414,7 +3414,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="874278767"/>
+        <c:crossAx val="1377578992"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3584,7 +3584,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6A38-4DD6-A2B8-E0175144CEA4}"/>
+              <c16:uniqueId val="{00000000-EBBA-4106-BDFD-553F7ABB8764}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3597,8 +3597,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1461339199"/>
-        <c:axId val="874267247"/>
+        <c:axId val="1442831616"/>
+        <c:axId val="1377575152"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -3720,7 +3720,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-6A38-4DD6-A2B8-E0175144CEA4}"/>
+              <c16:uniqueId val="{00000001-EBBA-4106-BDFD-553F7ABB8764}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3841,7 +3841,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-6A38-4DD6-A2B8-E0175144CEA4}"/>
+              <c16:uniqueId val="{00000002-EBBA-4106-BDFD-553F7ABB8764}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3962,7 +3962,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-6A38-4DD6-A2B8-E0175144CEA4}"/>
+              <c16:uniqueId val="{00000003-EBBA-4106-BDFD-553F7ABB8764}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4083,7 +4083,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-6A38-4DD6-A2B8-E0175144CEA4}"/>
+              <c16:uniqueId val="{00000004-EBBA-4106-BDFD-553F7ABB8764}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4160,7 +4160,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="874267247"/>
+        <c:axId val="1377575152"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4195,12 +4195,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1461339199"/>
+        <c:crossAx val="1442831616"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1461339199"/>
+        <c:axId val="1442831616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,7 +4210,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="874267247"/>
+        <c:crossAx val="1377575152"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -4380,7 +4380,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9C54-431B-8D7D-FF8E49F5CC0A}"/>
+              <c16:uniqueId val="{00000000-50A7-4FCB-AAE4-155A87FFBD81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4393,8 +4393,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1461334095"/>
-        <c:axId val="874266287"/>
+        <c:axId val="1442833472"/>
+        <c:axId val="1377569392"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4516,7 +4516,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9C54-431B-8D7D-FF8E49F5CC0A}"/>
+              <c16:uniqueId val="{00000001-50A7-4FCB-AAE4-155A87FFBD81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4637,7 +4637,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-9C54-431B-8D7D-FF8E49F5CC0A}"/>
+              <c16:uniqueId val="{00000002-50A7-4FCB-AAE4-155A87FFBD81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4758,7 +4758,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-9C54-431B-8D7D-FF8E49F5CC0A}"/>
+              <c16:uniqueId val="{00000003-50A7-4FCB-AAE4-155A87FFBD81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4879,7 +4879,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-9C54-431B-8D7D-FF8E49F5CC0A}"/>
+              <c16:uniqueId val="{00000004-50A7-4FCB-AAE4-155A87FFBD81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5000,7 +5000,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-9C54-431B-8D7D-FF8E49F5CC0A}"/>
+              <c16:uniqueId val="{00000005-50A7-4FCB-AAE4-155A87FFBD81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5077,7 +5077,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="874266287"/>
+        <c:axId val="1377569392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5112,12 +5112,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1461334095"/>
+        <c:crossAx val="1442833472"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1461334095"/>
+        <c:axId val="1442833472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5127,7 +5127,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="874266287"/>
+        <c:crossAx val="1377569392"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5297,7 +5297,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4765-4320-A9A7-50314BA64473}"/>
+              <c16:uniqueId val="{00000000-A0DC-4685-9046-397B8D0D78E3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5310,8 +5310,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1461335023"/>
-        <c:axId val="874279247"/>
+        <c:axId val="1436528352"/>
+        <c:axId val="1377571312"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5433,7 +5433,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4765-4320-A9A7-50314BA64473}"/>
+              <c16:uniqueId val="{00000001-A0DC-4685-9046-397B8D0D78E3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5554,7 +5554,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4765-4320-A9A7-50314BA64473}"/>
+              <c16:uniqueId val="{00000002-A0DC-4685-9046-397B8D0D78E3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5675,7 +5675,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-4765-4320-A9A7-50314BA64473}"/>
+              <c16:uniqueId val="{00000003-A0DC-4685-9046-397B8D0D78E3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5796,7 +5796,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-4765-4320-A9A7-50314BA64473}"/>
+              <c16:uniqueId val="{00000004-A0DC-4685-9046-397B8D0D78E3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5873,7 +5873,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="874279247"/>
+        <c:axId val="1377571312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5908,12 +5908,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1461335023"/>
+        <c:crossAx val="1436528352"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1461335023"/>
+        <c:axId val="1436528352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5923,7 +5923,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="874279247"/>
+        <c:crossAx val="1377571312"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6093,7 +6093,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6FC2-474F-ABD6-43C97DC86556}"/>
+              <c16:uniqueId val="{00000000-D284-4468-B2E2-B604EE5BDBDB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6106,8 +6106,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1461334559"/>
-        <c:axId val="874289327"/>
+        <c:axId val="1442830688"/>
+        <c:axId val="1377587632"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6229,7 +6229,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-6FC2-474F-ABD6-43C97DC86556}"/>
+              <c16:uniqueId val="{00000001-D284-4468-B2E2-B604EE5BDBDB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6350,7 +6350,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-6FC2-474F-ABD6-43C97DC86556}"/>
+              <c16:uniqueId val="{00000002-D284-4468-B2E2-B604EE5BDBDB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6471,7 +6471,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-6FC2-474F-ABD6-43C97DC86556}"/>
+              <c16:uniqueId val="{00000003-D284-4468-B2E2-B604EE5BDBDB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6592,7 +6592,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-6FC2-474F-ABD6-43C97DC86556}"/>
+              <c16:uniqueId val="{00000004-D284-4468-B2E2-B604EE5BDBDB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6669,7 +6669,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="874289327"/>
+        <c:axId val="1377587632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6704,12 +6704,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1461334559"/>
+        <c:crossAx val="1442830688"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1461334559"/>
+        <c:axId val="1442830688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6719,7 +6719,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="874289327"/>
+        <c:crossAx val="1377587632"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6889,7 +6889,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-348D-43F8-B337-7ECF132DED29}"/>
+              <c16:uniqueId val="{00000000-B141-4CB8-8252-704D0B7B2D52}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6902,8 +6902,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1461340127"/>
-        <c:axId val="874287887"/>
+        <c:axId val="1925784176"/>
+        <c:axId val="1377486832"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -7025,7 +7025,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-348D-43F8-B337-7ECF132DED29}"/>
+              <c16:uniqueId val="{00000001-B141-4CB8-8252-704D0B7B2D52}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7146,7 +7146,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-348D-43F8-B337-7ECF132DED29}"/>
+              <c16:uniqueId val="{00000002-B141-4CB8-8252-704D0B7B2D52}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7267,7 +7267,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-348D-43F8-B337-7ECF132DED29}"/>
+              <c16:uniqueId val="{00000003-B141-4CB8-8252-704D0B7B2D52}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7388,7 +7388,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-348D-43F8-B337-7ECF132DED29}"/>
+              <c16:uniqueId val="{00000004-B141-4CB8-8252-704D0B7B2D52}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7509,7 +7509,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-348D-43F8-B337-7ECF132DED29}"/>
+              <c16:uniqueId val="{00000005-B141-4CB8-8252-704D0B7B2D52}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7586,7 +7586,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="874287887"/>
+        <c:axId val="1377486832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -7621,12 +7621,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1461340127"/>
+        <c:crossAx val="1925784176"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1461340127"/>
+        <c:axId val="1925784176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7636,7 +7636,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="874287887"/>
+        <c:crossAx val="1377486832"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>

</xml_diff>